<commit_message>
Lead form value update
</commit_message>
<xml_diff>
--- a/public/templates/leads-import-template.xlsx
+++ b/public/templates/leads-import-template.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -482,9 +482,8 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -515,15 +514,10 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Assigned To Email</t>
         </is>
@@ -557,15 +551,10 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>15000</t>
+          <t>Met at the property expo, interested in a full inspection package</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Met at the property expo, interested in a full inspection package</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>mary@yourcompany.com</t>
         </is>
@@ -599,15 +588,10 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>8000</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
           <t>Requested a quote for a 3-bedroom unit</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -705,104 +689,104 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Value            - Optional. Estimated deal value, numbers only (e.g. 15000).</t>
+          <t xml:space="preserve">   Notes            - Optional. Any free-text notes.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Notes            - Optional. Any free-text notes.</t>
+          <t xml:space="preserve">   Assigned To Email- Optional. Must exactly match an existing admin/marketing team member's</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Assigned To Email- Optional. Must exactly match an existing admin/marketing team member's</t>
+          <t xml:space="preserve">                      login email. If left blank, or it doesn't match anyone, the lead is</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">                      login email. If left blank, or it doesn't match anyone, the lead is</t>
+          <t xml:space="preserve">                      assigned to whoever runs the import instead.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                      assigned to whoever runs the import instead.</t>
-        </is>
-      </c>
+      <c r="A17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr"/>
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>3. Importing into the app</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>3. Importing into the app</t>
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Option A - Upload this file directly (most reliable):</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Option A - Google Sheets (recommended):</t>
+          <t xml:space="preserve">     - In the app, go to Leads -&gt; Import Leads -&gt; Upload a CSV file, and select this file</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     - Upload this file to Google Drive and open it (it converts to a Google Sheet automatically),</t>
+          <t xml:space="preserve">       (or File &gt; Save As &gt; CSV from Excel/Sheets first).</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       or use File &gt; Import in an existing Google Sheet.</t>
-        </is>
-      </c>
+      <c r="A22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     - Click Share, and set sharing to "Anyone with the link" -&gt; Viewer.</t>
+          <t xml:space="preserve">   Option B - Google Sheets link:</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     - Copy the link and paste it into the app: Leads -&gt; Import from Google Sheets.</t>
+          <t xml:space="preserve">     - Upload this file to Google Drive and open it (it converts to a Google Sheet automatically).</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr"/>
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     - Click Share, and set sharing to "Anyone with the link" -&gt; Viewer.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Option B - Upload this file directly:</t>
+          <t xml:space="preserve">     - Copy the link and paste it into the app: Leads -&gt; Import Leads -&gt; paste the Google Sheets link.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     - In the app, go to Leads -&gt; Import from Google Sheets -&gt; Upload a CSV file instead,</t>
+          <t xml:space="preserve">     - Note: on Google Workspace/business accounts, this sometimes only shares within your</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">       and select this file (or File &gt; Save As &gt; CSV from Excel/Sheets first).</t>
+          <t xml:space="preserve">       organization even when it looks public. If that happens, use Option A instead.</t>
         </is>
       </c>
     </row>

</xml_diff>